<commit_message>
docs: Add Bug 6 (Quotes-only Policy Name Defect) to all bug sheets and reports
</commit_message>
<xml_diff>
--- a/reports/HCM_API_Bug_Sheet_17Aug2026.xlsx
+++ b/reports/HCM_API_Bug_Sheet_17Aug2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="52">
   <si>
     <t>Bug ID</t>
   </si>
@@ -157,6 +157,24 @@
   </si>
   <si>
     <t>Add @DecimalMin(value = '0.00') and @DecimalMax(value = '24.00') constraint annotations across all threshold hour fields</t>
+  </si>
+  <si>
+    <t>BUG-HCM-ATT-006</t>
+  </si>
+  <si>
+    <t>Late / Early Policy Master</t>
+  </si>
+  <si>
+    <t>Missing Input Validation for Special-Character-Only Values in Policy Name (Accepted quotes-only Name)</t>
+  </si>
+  <si>
+    <t>/api/attendance/late-early-policies/create</t>
+  </si>
+  <si>
+    <t>DTO lacks regex pattern validation on policyName; persists quotes-only string</t>
+  </si>
+  <si>
+    <t>Add @NotBlank and @Pattern(regexp = '^(?=.*[a-zA-Z0-9])[a-zA-Z0-9\s\-_/().]+$') on policyName</t>
   </si>
 </sst>
 </file>
@@ -970,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -1215,6 +1233,44 @@
         <v>23</v>
       </c>
     </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: Add Bug 7 (Unhandled 500 JPA Entity Leak on Sort) to all bug sheets
</commit_message>
<xml_diff>
--- a/reports/HCM_API_Bug_Sheet_17Aug2026.xlsx
+++ b/reports/HCM_API_Bug_Sheet_17Aug2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="56">
   <si>
     <t>Bug ID</t>
   </si>
@@ -175,6 +175,18 @@
   </si>
   <si>
     <t>Add @NotBlank and @Pattern(regexp = '^(?=.*[a-zA-Z0-9])[a-zA-Z0-9\s\-_/().]+$') on policyName</t>
+  </si>
+  <si>
+    <t>BUG-HCM-ATT-007</t>
+  </si>
+  <si>
+    <t>Unhandled 500 Internal Server Error &amp; JPA Entity Leak on Invalid Sort Query Parameter</t>
+  </si>
+  <si>
+    <t>/api/attendance/late-early-policies/getAll?sort=non_existent_column,desc</t>
+  </si>
+  <si>
+    <t>Spring Data JPA throws unhandled PropertyReferenceException; leaks 'LateEarlyPolicyMaster' entity name</t>
   </si>
 </sst>
 </file>
@@ -988,7 +1000,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -997,7 +1009,7 @@
     <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="68.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="69.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="115.5703125" bestFit="1" customWidth="1"/>
@@ -1271,6 +1283,44 @@
         <v>23</v>
       </c>
     </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: Add Bug 9 (Inactive Leave Type Gating & UI Edit Failure) with full navigation
</commit_message>
<xml_diff>
--- a/reports/HCM_API_Bug_Sheet_17Aug2026.xlsx
+++ b/reports/HCM_API_Bug_Sheet_17Aug2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="68">
   <si>
     <t>Bug ID</t>
   </si>
@@ -211,6 +211,18 @@
   </si>
   <si>
     <t>In changeStatus(), execute cascade update: assignmentRepository.updateStatusByPolicyId(policyId, newStatus)</t>
+  </si>
+  <si>
+    <t>BUG-HCM-ATT-009</t>
+  </si>
+  <si>
+    <t>Missing Foreign Active-State Validation on Leave Type Allows Linking Deactivated Leaves (UI Rendering &amp; Edit Failure)</t>
+  </si>
+  <si>
+    <t>Service layer checks leaveTypeId existence but ignores is_active == 'Y' flag; creates un-editable UI policies</t>
+  </si>
+  <si>
+    <t>Validate leaveType.getIsActive().equals('Y') before saving policy</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -1383,6 +1395,44 @@
         <v>23</v>
       </c>
     </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" t="s">
+        <v>66</v>
+      </c>
+      <c r="K10" t="s">
+        <v>67</v>
+      </c>
+      <c r="L10" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>